<commit_message>
v1.4.0 server / v1.5.0 HHT: FG parts flow, PDI, WMS stock, internal movement, missed scans
- Dispatch types: customer / stock transfer (EBS invoice), empty return (EBS challan + e-way bill), pallets only
- Blanket order master controls PO + schedule; SO pushed to EBS only after PDI
- PDI per LPN; EBS sub-inventory transfer with double confirmation
- WMS stock upload / EBS pull with freshness gate; in-process LPNs protected; reservation control
- Dock scan: LPN fetches pallet, pallet fetches all LPNs
- Loaded / empty state; in-plant zones and internal movement; Yard = empty only
- Other-plant material receipt at FGWH / Packing
- Missed-scan detection, alerts, auto-correct, register
- Auto DB upgrade; end-to-end regression test (41 checks)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4tKsFhnpMECYWmxddZRvd
</commit_message>
<xml_diff>
--- a/docs/Pallet_Tracking_Master_Template_v0.4.xlsx
+++ b/docs/Pallet_Tracking_Master_Template_v0.4.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Transporters" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Pallets" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Tags" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Blanket_Orders" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_SubInv_Rules" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -633,13 +635,155 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Plant_Code</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Customer_Code</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Part_No</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>OK_SubInv</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>OK_Locator</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Reject_SubInv</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Plant</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Blank = any customer</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Blank = any part</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>PDI OK -&gt; this sub-inventory</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Optional locator</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>PDI reject -&gt; this sub-inventory</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Y/N</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>EXAMPLE row is skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CHN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HMIL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HMIL-FG</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>REJ</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:T53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -659,6 +803,9 @@
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -747,6 +894,21 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>WMS_Stale_Hours</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>PDI_SubInv</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>Reject_SubInv</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
@@ -822,6 +984,21 @@
         </is>
       </c>
       <c r="Q2" s="6" t="inlineStr"/>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>Block release if WMS stock older (hours), default 4</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>Sub-inventory where picked LPNs wait for PDI (optional)</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>PDI rejected LPNs go here, e.g. REJ</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -7165,4 +7342,228 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Plant_Code</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Customer_Code</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Part_No</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Customer_Part_No</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Blanket_No</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>PO_Number</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Schedule_Qty</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Valid_From</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Valid_To</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Dispatch_Type</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>To_Plant</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Dispatching plant</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Customer code (stock transfer: receiving plant code)</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>AIS item code</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Customer item code</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Customer blanket / scheduling agreement</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>PO number printed on SO</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Total schedule qty</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>dd-mm-yyyy</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>dd-mm-yyyy</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>CUSTOMER or STOCK_TRANSFER</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Stock transfer destination plant</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Y/N</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>EXAMPLE row is skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CHN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HMIL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WS-1234-FR</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>86110-XX000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BL-2026-01</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4500012345</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>01-10-2026</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>31-03-2027</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CUSTOMER</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>